<commit_message>
feat(release): prepare Dauam TestFlight build 12
</commit_message>
<xml_diff>
--- a/Jadwal — сбор зикров.xlsx
+++ b/Jadwal — сбор зикров.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R7d8d386364fe4e3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Зикры" sheetId="2" r:id="R2b08bc81e3544cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R1edc5c4a32fb42c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Зикры" sheetId="2" r:id="Rf439e04b6ac74500"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -802,7 +802,7 @@
         <x:v>اللَّهُمَّ إِنِّي أَصْبَحْتُ أُشْهِدُكَ وَأُشْهِدُ حَمَلَةَ عَرْشِكَ وَمَلَائِكَتَكَ وَجَمِيعَ خَلْقِكَ، أَنَّكَ أَنْتَ اللَّهُ لَا إِلَهَ إِلَّا أَنْتَ وَحْدَكَ لَا شَرِيكَ لَكَ، وَأَنَّ مُحَمَّدًا عَبْدُكَ وَرَسُولُكَ</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
-        <x:v>Аллахумма инни асбахту (вечером: амсайту) уш-хидука ва уш-хиду хамалята 'аршик, ва маляикатак, ва джами'а халькик…</x:v>
+        <x:v>Аллахумма инни асбахту ушхиду-ка ва ушхиду хамалята ‘арши-ка ва маля’иката-ка ва джами‘а халькы-ка анна-ка анта Ллаху ля иляха илля анта вахда-ка ля шарика ля-ка ва анна Мухаммадан ‘абду-ка ва расулю-ка.</x:v>
       </x:c>
       <x:c r="E7" s="6" t="str">
         <x:v>«О Аллах, я встретил утро, призывая в свидетели Тебя, носителей Твоего Трона, Твоих ангелов и всё Твоё творение, что Ты — Аллах, нет божества, кроме Тебя, и что Мухаммад — Твой раб и посланник».</x:v>
@@ -1675,7 +1675,7 @@
         <x:v>اللَّهُمَّ إِنِّي أَمْسَيْتُ أُشْهِدُكَ وَأُشْهِدُ حَمَلَةَ عَرْشِكَ وَمَلَائِكَتَكَ وَجَمِيعَ خَلْقِكَ، أَنَّكَ أَنْتَ اللَّهُ لَا إِلَهَ إِلَّا أَنْتَ وَحْدَكَ لَا شَرِيكَ لَكَ، وَأَنَّ مُحَمَّدًا عَبْدُكَ وَرَسُولُكَ</x:v>
       </x:c>
       <x:c r="D30" s="6" t="str">
-        <x:v>Аллахумма инни асбахту (вечером: амсайту) уш-хидука ва уш-хиду хамалята 'аршик, ва маляикатак, ва джами'а халькик…</x:v>
+        <x:v>Аллахумма инни амсайту ушхиду-ка ва ушхиду хамалята ‘арши-ка ва маля’иката-ка ва джами‘а халькы-ка анна-ка анта Ллаху ля иляха илля анта вахда-ка ля шарика ля-ка ва анна Мухаммадан ‘абду-ка ва расулю-ка.</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
         <x:v>«О Аллах, я встретил утро, призывая в свидетели Тебя, носителей Твоего Трона, Твоих ангелов и всё Твоё творение, что Ты — Аллах, нет божества, кроме Тебя, и что Мухаммад — Твой раб и посланник».</x:v>

</xml_diff>